<commit_message>
Remove Priority column from the Import Projects template
The app's import validation stopped checking Priority when Commitment
replaced it, but the downloadable .xlsx template still had the column,
its example value, its dropdown validation, and a mention in the
instructions -- all removed now, with every column after it shifted
left and column widths preserved.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pmo-hub-project-import-template.xlsx
+++ b/pmo-hub-project-import-template.xlsx
@@ -1,21 +1,45 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">openpyxl</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-30T20:08:50Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-08-03T23:53:28Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\comments\comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>PMO Hub</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Leave this blank in almost every case -- PMO Hub derives Backlog/Planned/Active automatically from Start Date and Target End Date. Only enter Hold or Complete here, to mark a project as already paused or finished (something dates alone can not show).</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it is shown as text only.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it's shown as text only.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="5">
@@ -161,32 +185,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>PMO Hub</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Leave this blank in almost every case -- PMO Hub derives Backlog/Planned/Active automatically from Start Date and Target End Date. Only enter Hold or Complete here, to mark a project as already paused or finished (something dates alone can not show).</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it is shown as text only.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>If this email matches an existing PMO Hub account, the project will be linked to that person for permissions. Otherwise it's shown as text only.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -469,7 +468,23 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="2" state="visible" r:id="rId2"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -515,7 +530,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Columns with a dropdown arrow (Business Unit, Status, Phase, Priority, Value Area)</t>
+          <t>3. Columns with a dropdown arrow (Business Unit, Status, Phase, Value Area)</t>
         </is>
       </c>
     </row>
@@ -623,13 +638,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -640,14 +655,13 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -693,40 +707,35 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Value Area</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>Value Area</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Target End Date</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>Target End Date</t>
+          <t>Progress %</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
-          <t>Progress %</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Current Blockers</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>Current Blockers</t>
-        </is>
-      </c>
-      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
@@ -770,45 +779,40 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Operational Efficiency</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Operational Efficiency</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>35</v>
       </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Automating pallet routing in the East distribution center.</t>
+        </is>
+      </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>Automating pallet routing in the East distribution center.</t>
+          <t>Waiting on hardware vendor lead time</t>
         </is>
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>Waiting on hardware vendor lead time</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
           <t>Supply Chain, CRM System</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="E3:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Customer Experience,Finance,Legal &amp; Compliance,Marketing,Operations,Product,Sales,Supply Chain,Technology"</formula1>
     </dataValidation>
@@ -819,9 +823,6 @@
       <formula1>"Not Started,On Track,At Risk,Planning,Blocked,Complete"</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,High,Medium,Low,Needs prioritization"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J3:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Revenue Growth,Customer Experience,Operational Efficiency,Employee Experience,Compliance &amp; Risk"</formula1>
     </dataValidation>
     <dataValidation sqref="H3:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>